<commit_message>
modifiny (.env) (setting.py) (docker-compose.yml).
</commit_message>
<xml_diff>
--- a/nodes.xlsx
+++ b/nodes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\myProjects\structural-analysis-app-v4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E1E48D2-C188-42A0-8BC9-B99B9F733A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC30E3CA-E238-43E5-B7F9-1705C2759FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17175" yWindow="105" windowWidth="15735" windowHeight="20775" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24300" yWindow="660" windowWidth="15540" windowHeight="15615" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,15 +25,138 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>y</t>
-  </si>
-  <si>
-    <t>z</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>services</t>
+  </si>
+  <si>
+    <t>volumes</t>
+  </si>
+  <si>
+    <t>db</t>
+  </si>
+  <si>
+    <t>backend</t>
+  </si>
+  <si>
+    <t>frontend</t>
+  </si>
+  <si>
+    <t>image</t>
+  </si>
+  <si>
+    <t>container_name</t>
+  </si>
+  <si>
+    <t>restart</t>
+  </si>
+  <si>
+    <t>environment</t>
+  </si>
+  <si>
+    <t>MYSQL_DATABASE</t>
+  </si>
+  <si>
+    <t>MYSQL_USER</t>
+  </si>
+  <si>
+    <t>MYSQL_PASSWORD</t>
+  </si>
+  <si>
+    <t>MYSQL_ROOT_PASSWORD</t>
+  </si>
+  <si>
+    <t>ports</t>
+  </si>
+  <si>
+    <t>build</t>
+  </si>
+  <si>
+    <t>command</t>
+  </si>
+  <si>
+    <t>depends_on</t>
+  </si>
+  <si>
+    <t>DB_HOST</t>
+  </si>
+  <si>
+    <t>DB_PORT</t>
+  </si>
+  <si>
+    <t>DB_NAME</t>
+  </si>
+  <si>
+    <t>DB_USER</t>
+  </si>
+  <si>
+    <t>DB_PASSWORD</t>
+  </si>
+  <si>
+    <t>context</t>
+  </si>
+  <si>
+    <t>dockerfile</t>
+  </si>
+  <si>
+    <t>db_data</t>
+  </si>
+  <si>
+    <t>3.9'</t>
+  </si>
+  <si>
+    <t>mysql:8.0</t>
+  </si>
+  <si>
+    <t>structural-db</t>
+  </si>
+  <si>
+    <t>always</t>
+  </si>
+  <si>
+    <t>space_truss_db_v4</t>
+  </si>
+  <si>
+    <t>space_truss_db_v4_user</t>
+  </si>
+  <si>
+    <t>root</t>
+  </si>
+  <si>
+    <t>"3311:3306"</t>
+  </si>
+  <si>
+    <t>db_data:/var/lib/mysql</t>
+  </si>
+  <si>
+    <t>./backend</t>
+  </si>
+  <si>
+    <t>Dockerfile.backend</t>
+  </si>
+  <si>
+    <t>structural-backend</t>
+  </si>
+  <si>
+    <t>./backend:/app</t>
+  </si>
+  <si>
+    <t>"8000:8000"</t>
+  </si>
+  <si>
+    <t>./frontend</t>
+  </si>
+  <si>
+    <t>Dockerfile.frontend</t>
+  </si>
+  <si>
+    <t>structural-frontend</t>
+  </si>
+  <si>
+    <t>"5173:80"</t>
   </si>
 </sst>
 </file>
@@ -49,15 +172,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -65,12 +194,130 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -351,65 +598,344 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C5:E9"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="9.140625" style="9"/>
+    <col min="3" max="3" width="15.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="9"/>
+  </cols>
   <sheetData>
-    <row r="5" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C5" t="s">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E1" s="17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E5" t="s">
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="10"/>
+      <c r="E2" s="18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="11"/>
+      <c r="E3" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="11"/>
+      <c r="E4" s="18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="18">
+        <v>9348</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="E9" s="18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="11" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C7">
-        <v>50</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C8">
-        <v>100</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C9">
-        <v>50</v>
-      </c>
-      <c r="D9">
-        <v>100</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
+      <c r="D10" s="11"/>
+      <c r="E10" s="18" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+      <c r="B11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="11"/>
+      <c r="E13" s="18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="11"/>
+      <c r="E14" s="18"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="11"/>
+      <c r="E15" s="18" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="11"/>
+      <c r="E17" s="18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="18">
+        <v>3306</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="1"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" s="18">
+        <v>9348</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="11"/>
+      <c r="E25" s="18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="11"/>
+      <c r="E26" s="18" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="1"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="12"/>
+      <c r="E27" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A2:A27"/>
+    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="B2:B10"/>
+    <mergeCell ref="B11:B22"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="C18:C22"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="B23:B27"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>